<commit_message>
Harden admin uploads and align mobile and topic config
</commit_message>
<xml_diff>
--- a/infra/test_upload.xlsx
+++ b/infra/test_upload.xlsx
@@ -484,7 +484,7 @@
         <v>Auto</v>
       </c>
       <c r="B2" t="str">
-        <v>Select ▼</v>
+        <v>Select v</v>
       </c>
       <c r="C2" t="str">
         <v/>
@@ -520,13 +520,13 @@
         <v>e.g. 1</v>
       </c>
       <c r="N2" t="str">
-        <v>Select ▼</v>
+        <v>Select v</v>
       </c>
       <c r="O2" t="str">
         <v>Yes / No</v>
       </c>
       <c r="P2" t="str">
-        <v>Select ▼</v>
+        <v>Select v</v>
       </c>
       <c r="Q2" t="str">
         <v>Use exact code</v>
@@ -535,13 +535,13 @@
         <v>Use exact code</v>
       </c>
       <c r="S2" t="str">
-        <v>Select ▼</v>
+        <v>Select v</v>
       </c>
       <c r="T2" t="str">
-        <v>Select ▼</v>
+        <v>Select v</v>
       </c>
       <c r="U2" t="str">
-        <v>Select ▼</v>
+        <v>Select v</v>
       </c>
       <c r="V2" t="str">
         <v>e.g. 2022</v>
@@ -573,7 +573,7 @@
         <v>Section A</v>
       </c>
       <c r="E3" t="str">
-        <v>Which of the following is the value of 3² + 4²?</v>
+        <v>Which of the following is the value of 3^2 + 4^2?</v>
       </c>
       <c r="F3" t="str">
         <v/>
@@ -594,7 +594,7 @@
         <v>C</v>
       </c>
       <c r="L3" t="str">
-        <v>3²=9 and 4²=16. Therefore 3²+4²=25.</v>
+        <v>3^2 = 9 and 4^2 = 16. Therefore 3^2 + 4^2 = 25.</v>
       </c>
       <c r="M3">
         <v>1</v>
@@ -612,7 +612,7 @@
         <v>MATH-JCE</v>
       </c>
       <c r="R3" t="str">
-        <v>MATH-JCE-NUMBERS</v>
+        <v>MATH-JCE-NUMBERS-SETS-AND-NUMBER-SYSTEMS</v>
       </c>
       <c r="S3" t="str">
         <v>MANEB Past Paper</v>
@@ -692,7 +692,7 @@
         <v>BIOL-JCE</v>
       </c>
       <c r="R4" t="str">
-        <v>BIOL-JCE-CELLS</v>
+        <v>BIOL-JCE-CELL-STRUCTURE-AND-FUNCTION</v>
       </c>
       <c r="S4" t="str">
         <v>MANEB Past Paper</v>
@@ -754,7 +754,7 @@
         <v>C</v>
       </c>
       <c r="L5" t="str">
-        <v>x = 15 − 7 = 8.</v>
+        <v>x = 15 - 7 = 8.</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -772,7 +772,7 @@
         <v>MATH-JCE</v>
       </c>
       <c r="R5" t="str">
-        <v>MATH-JCE-NUMBERS</v>
+        <v>MATH-JCE-NUMBERS-SETS-AND-NUMBER-SYSTEMS</v>
       </c>
       <c r="S5" t="str">
         <v>Teacher Created</v>

</xml_diff>